<commit_message>
Add Pattern C navbar to notifications page, add email notification service
</commit_message>
<xml_diff>
--- a/publisher_test_checklist.xlsx
+++ b/publisher_test_checklist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\test-publishing-platform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDD6521-7C8A-4C01-892F-6239481653E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121B2B58-FD11-4E2F-B50B-CE9D662C81DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12840" yWindow="2835" windowWidth="15960" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="132">
   <si>
     <t>#</t>
   </si>
@@ -1086,9 +1086,15 @@
       <c r="E8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="F8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="I8" s="2" t="s">
         <v>8</v>
       </c>
@@ -1112,9 +1118,15 @@
       <c r="E9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="F9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="I9" s="2" t="s">
         <v>8</v>
       </c>
@@ -1170,9 +1182,15 @@
       <c r="E11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="F11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="I11" s="2" t="s">
         <v>8</v>
       </c>
@@ -1196,9 +1214,15 @@
       <c r="E12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
+      <c r="F12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="I12" s="2" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Clean up: Update backend configs, remove deprecated pages
- Update backend email, payments, receipt-generator configs
- Remove deprecated pages: analytics, index (pages/), manga-viewer,
  register-translator, terms_with_zh, upload-work, portuguese_translation,
  privacy duplicates (privacy.html, privacy_complete/final/updated.html)
- Update project documentation

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/publisher_test_checklist.xlsx
+++ b/publisher_test_checklist.xlsx
@@ -8,21 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\test-publishing-platform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121B2B58-FD11-4E2F-B50B-CE9D662C81DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89FB85BB-EB8B-46B2-BFBB-ECF8A959253A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12840" yWindow="2835" windowWidth="15960" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="15960" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="テストチェックリスト" sheetId="1" r:id="rId1"/>
     <sheet name="凡例" sheetId="2" r:id="rId2"/>
     <sheet name="チェック記入方法" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="137">
   <si>
     <t>#</t>
   </si>
@@ -418,13 +429,103 @@
   </si>
   <si>
     <t>翻訳機能</t>
+  </si>
+  <si>
+    <t>アカウントマークをつける</t>
+  </si>
+  <si>
+    <t>アカウントマークつける</t>
+  </si>
+  <si>
+    <t>この要件は現在のcontact.htmlのフォームに「Data Protection Complaint」カテゴリを追加し、30日以内の確認応答プロセスを整備する</t>
+  </si>
+  <si>
+    <r>
+      <t>要確認</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> イギリスでは </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>UK GDPR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> と </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Protection Act 2018</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">（さらに2025年施行の </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data (Use and Access) Act 2025</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>）が適用されます。Privacy Policyの方をこれらに準拠させる必要があり/ Analytics Cookieのプロバイダーは未定</t>
+    </r>
+  </si>
+  <si>
+    <t>18+ やAI、過度な暴力、センシティブなトピック、教育的・芸術的な目的であることの表示をするための項目はあるか？</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -437,6 +538,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -472,7 +581,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -495,11 +604,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -529,6 +664,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -907,7 +1049,7 @@
         <v>8</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>9</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -939,7 +1081,7 @@
         <v>8</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>9</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -1118,9 +1260,7 @@
       <c r="E9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
         <v>8</v>
       </c>
@@ -1150,9 +1290,7 @@
       <c r="E10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
         <v>8</v>
       </c>
@@ -1182,9 +1320,7 @@
       <c r="E11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
         <v>8</v>
       </c>
@@ -1214,9 +1350,7 @@
       <c r="E12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
         <v>8</v>
       </c>
@@ -1279,7 +1413,7 @@
         <v>8</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>9</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -1305,7 +1439,7 @@
         <v>8</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>9</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -1324,9 +1458,15 @@
       <c r="E16" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="F16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="I16" s="2" t="s">
         <v>8</v>
       </c>
@@ -1350,9 +1490,15 @@
       <c r="E17" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
+      <c r="F17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="I17" s="2" t="s">
         <v>8</v>
       </c>
@@ -1373,13 +1519,19 @@
       <c r="D18" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I18" s="10" t="s">
+      <c r="G18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J18" t="s">
@@ -1396,15 +1548,27 @@
       <c r="C19" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J19" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="20" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
@@ -1416,15 +1580,27 @@
       <c r="C20" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
+      <c r="E20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="21" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
@@ -1439,12 +1615,24 @@
       <c r="D21" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
+      <c r="E21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J21" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="22" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
@@ -1459,12 +1647,24 @@
       <c r="D22" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
+      <c r="E22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="23" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
@@ -1479,12 +1679,24 @@
       <c r="D23" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
+      <c r="E23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J23" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="24" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
@@ -1499,12 +1711,24 @@
       <c r="D24" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
+      <c r="E24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="25" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
@@ -1519,12 +1743,24 @@
       <c r="D25" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
+      <c r="E25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="26" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
@@ -1539,12 +1775,24 @@
       <c r="D26" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
+      <c r="E26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="27" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
@@ -1559,12 +1807,24 @@
       <c r="D27" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
+      <c r="E27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J27" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="28" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
@@ -1579,12 +1839,24 @@
       <c r="D28" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
+      <c r="E28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="29" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
@@ -1599,12 +1871,24 @@
       <c r="D29" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
+      <c r="E29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J29" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
@@ -1619,12 +1903,24 @@
       <c r="D30" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
+      <c r="E30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="31" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
@@ -1639,12 +1935,24 @@
       <c r="D31" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
+      <c r="E31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J31" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
@@ -1659,12 +1967,24 @@
       <c r="D32" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
+      <c r="E32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
@@ -1679,12 +1999,24 @@
       <c r="D33" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
+      <c r="E33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J33" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="34" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
@@ -1699,12 +2031,24 @@
       <c r="D34" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
+      <c r="E34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J34" s="13" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="35" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
@@ -1719,12 +2063,24 @@
       <c r="D35" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
+      <c r="E35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J35" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="36" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
@@ -1739,12 +2095,24 @@
       <c r="D36" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
+      <c r="E36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J36" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
@@ -1759,12 +2127,24 @@
       <c r="D37" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
+      <c r="E37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J37" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="38" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2">

</xml_diff>